<commit_message>
data(nzd): all refresh 2026-10-01T11:29Z
</commit_message>
<xml_diff>
--- a/logs/nzd/raw/C5.xlsx
+++ b/logs/nzd/raw/C5.xlsx
@@ -23408,6 +23408,65 @@
         <v>2.4</v>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" s="28">
+        <v>46265</v>
+      </c>
+      <c r="B434" s="16">
+        <v>403342</v>
+      </c>
+      <c r="C434" s="16">
+        <v>398235</v>
+      </c>
+      <c r="D434" s="16">
+        <v>5107</v>
+      </c>
+      <c r="E434" s="16">
+        <v>14561</v>
+      </c>
+      <c r="F434" s="16">
+        <v>7285</v>
+      </c>
+      <c r="G434" s="16">
+        <v>7276</v>
+      </c>
+      <c r="H434" s="16">
+        <v>417903</v>
+      </c>
+      <c r="I434" s="16">
+        <v>405520</v>
+      </c>
+      <c r="J434" s="16">
+        <v>12383</v>
+      </c>
+      <c r="K434" s="16">
+        <v>143781</v>
+      </c>
+      <c r="L434" s="16">
+        <v>133949</v>
+      </c>
+      <c r="M434" s="16">
+        <v>9832</v>
+      </c>
+      <c r="N434" s="16">
+        <v>65655</v>
+      </c>
+      <c r="O434" s="10">
+        <v>5.5</v>
+      </c>
+      <c r="P434" s="10">
+        <v>2.2</v>
+      </c>
+      <c r="Q434" s="10">
+        <v>5.4</v>
+      </c>
+      <c r="R434" s="10">
+        <v>4.1</v>
+      </c>
+      <c r="S434" s="10">
+        <v>2.4</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B5" location="'Series Definitions'!R2C3"/>
@@ -23471,7 +23530,7 @@
         <v>54</v>
       </c>
       <c r="B4" s="27">
-        <v>46265</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="5"/>

</xml_diff>